<commit_message>
fixed teacher timetable bug
</commit_message>
<xml_diff>
--- a/uploads/lab_rooms.xlsx
+++ b/uploads/lab_rooms.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D96B92E9-F35B-4AB9-8DA9-F1BDF1FE6C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC475C51-BFBA-495C-935E-0EDD1EBE3AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C81C6726-5086-4F86-A491-46F0D6D31795}"/>
   </bookViews>
@@ -281,9 +281,6 @@
     <t>A401B,A402B</t>
   </si>
   <si>
-    <t>A401B,A</t>
-  </si>
-  <si>
     <t>A401,A205</t>
   </si>
   <si>
@@ -294,6 +291,9 @@
   </si>
   <si>
     <t>A,A507</t>
+  </si>
+  <si>
+    <t>A401B,A507</t>
   </si>
 </sst>
 </file>
@@ -786,7 +786,7 @@
         <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -797,7 +797,7 @@
         <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -819,7 +819,7 @@
         <v>54</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -852,7 +852,7 @@
         <v>68</v>
       </c>
       <c r="C15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -863,7 +863,7 @@
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1006,7 +1006,7 @@
         <v>49</v>
       </c>
       <c r="C29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1017,7 +1017,7 @@
         <v>49</v>
       </c>
       <c r="C30" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1083,7 +1083,7 @@
         <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>